<commit_message>
feat: Update project KPIs and sprint review documentation, including sprint metrics and backlog adjustments
</commit_message>
<xml_diff>
--- a/docs/tecnico/OnBoardPro-Backlog.xlsx
+++ b/docs/tecnico/OnBoardPro-Backlog.xlsx
@@ -275,12 +275,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Métricas por sprint'!$A$2:$A$7</f>
+              <f>'Métricas por sprint'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Métricas por sprint'!$G$2:$G$7</f>
+              <f>'Métricas por sprint'!$G$2:$G$8</f>
             </numRef>
           </val>
         </ser>
@@ -299,12 +299,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Métricas por sprint'!$A$2:$A$7</f>
+              <f>'Métricas por sprint'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Métricas por sprint'!$H$2:$H$7</f>
+              <f>'Métricas por sprint'!$H$2:$H$8</f>
             </numRef>
           </val>
         </ser>
@@ -419,12 +419,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Métricas por sprint'!$A$2:$A$7</f>
+              <f>'Métricas por sprint'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Métricas por sprint'!$J$2:$J$7</f>
+              <f>'Métricas por sprint'!$J$2:$J$8</f>
             </numRef>
           </val>
         </ser>
@@ -451,12 +451,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Métricas por sprint'!$A$2:$A$7</f>
+              <f>'Métricas por sprint'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Métricas por sprint'!$K$2:$K$7</f>
+              <f>'Métricas por sprint'!$K$2:$K$8</f>
             </numRef>
           </val>
         </ser>
@@ -563,12 +563,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Métricas por sprint'!$A$2:$A$7</f>
+              <f>'Métricas por sprint'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Métricas por sprint'!$L$2:$L$7</f>
+              <f>'Métricas por sprint'!$L$2:$L$8</f>
             </numRef>
           </val>
         </ser>
@@ -7860,23 +7860,33 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="E8" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="F8" s="11" t="n"/>
+      <c r="F8" s="11" t="n">
+        <v>7</v>
+      </c>
       <c r="G8" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="H8" s="11" t="n"/>
-      <c r="I8" s="13" t="n"/>
-      <c r="J8" s="11" t="n"/>
+      <c r="H8" s="11" t="n">
+        <v>27</v>
+      </c>
+      <c r="I8" s="13" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J8" s="11" t="n">
+        <v>130</v>
+      </c>
       <c r="K8" s="11" t="n">
         <v>226</v>
       </c>
-      <c r="L8" s="11" t="n"/>
+      <c r="L8" s="11" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
@@ -8032,28 +8042,28 @@
       <c r="C13" s="11" t="inlineStr"/>
       <c r="D13" s="11" t="inlineStr"/>
       <c r="E13" s="11" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>109</v>
+        <v>139</v>
       </c>
       <c r="H13" s="11" t="n">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="I13" s="13" t="n">
-        <v>0.945</v>
+        <v>0.9353</v>
       </c>
       <c r="J13" s="11" t="n">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="K13" s="11" t="n">
         <v>226</v>
       </c>
       <c r="L13" s="11" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -8527,7 +8537,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Sprint 6 · 2026-10-09</t>
+          <t>Sprint 7 · 2026-10-16</t>
         </is>
       </c>
     </row>
@@ -8555,7 +8565,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>6 de 11</t>
+          <t>7 de 11</t>
         </is>
       </c>
     </row>
@@ -8567,7 +8577,7 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>103 de 226 SP · 46%</t>
+          <t>130 de 226 SP · 58%</t>
         </is>
       </c>
     </row>
@@ -8579,7 +8589,7 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>32 de 34</t>
+          <t>39 de 42</t>
         </is>
       </c>
     </row>
@@ -8591,7 +8601,7 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>17.2 SP</t>
+          <t>18.6 SP</t>
         </is>
       </c>
     </row>
@@ -8603,7 +8613,7 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>19.7 SP</t>
+          <t>23.0 SP</t>
         </is>
       </c>
     </row>
@@ -8615,7 +8625,7 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>94% · 103 de 109 SP</t>
+          <t>94% · 130 de 139 SP</t>
         </is>
       </c>
     </row>
@@ -8627,7 +8637,7 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>123 en 5 sprints</t>
+          <t>96 en 4 sprints</t>
         </is>
       </c>
     </row>
@@ -8695,7 +8705,7 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>0.12 por SP entregado</t>
+          <t>0.09 por SP entregado</t>
         </is>
       </c>
     </row>

</xml_diff>